<commit_message>
docs(audit): refresh final compliance report
Record the 15 August audit run after formula and repository synchronization. The report contains 208 passes, no failures, two author actions, and two external preview checks.

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/submission_documents/audits/Journal_of_Cheminformatics_full_audit_20260815.xlsx
+++ b/submission_documents/audits/Journal_of_Cheminformatics_full_audit_20260815.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="File inventory" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$E$211</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'File inventory'!$A$1:$E$150</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$E$213</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'File inventory'!$A$1:$E$154</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -466,7 +466,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-15</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>149</v>
+        <v>153</v>
       </c>
     </row>
     <row r="4">
@@ -551,7 +551,7 @@
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>206</v>
+        <v>208</v>
       </c>
     </row>
   </sheetData>
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E211"/>
+  <dimension ref="A1:E213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -4560,12 +4560,12 @@
       </c>
       <c r="C173" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: full_content_and_format_consistency_audit.xlsx</t>
+          <t>No Excel error tokens: formula_table_and_format_audit_20260815.xlsx</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
         <is>
-          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E173" s="2" t="inlineStr"/>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C174" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: journal_format_compliance_audit.xlsx</t>
+          <t>No Excel error tokens: full_content_and_format_consistency_audit.xlsx</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -4606,12 +4606,12 @@
       </c>
       <c r="C175" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: Journal_of_Cheminformatics_full_submission_audit_20260810.xlsx</t>
+          <t>No Excel error tokens: journal_format_compliance_audit.xlsx</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
         <is>
-          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E175" s="2" t="inlineStr"/>
@@ -4629,12 +4629,12 @@
       </c>
       <c r="C176" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: Figure_6_source_data.xlsx</t>
+          <t>No Excel error tokens: Journal_of_Cheminformatics_full_audit_20260815.xlsx</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
         <is>
-          <t>sheets=4; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E176" s="2" t="inlineStr"/>
@@ -4652,12 +4652,12 @@
       </c>
       <c r="C177" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: matched_stochastic_registry_results.xlsx</t>
+          <t>No Excel error tokens: Journal_of_Cheminformatics_full_submission_audit_20260810.xlsx</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
         <is>
-          <t>sheets=4; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E177" s="2" t="inlineStr"/>
@@ -4675,12 +4675,12 @@
       </c>
       <c r="C178" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: metric_recomputation_report.xlsx</t>
+          <t>No Excel error tokens: Figure_6_source_data.xlsx</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
         <is>
-          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=4; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E178" s="2" t="inlineStr"/>
@@ -4698,12 +4698,12 @@
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: model_seed_design_audit.xlsx</t>
+          <t>No Excel error tokens: matched_stochastic_registry_results.xlsx</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
         <is>
-          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=4; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E179" s="2" t="inlineStr"/>
@@ -4721,7 +4721,7 @@
       </c>
       <c r="C180" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: model_seed_results_revised.xlsx</t>
+          <t>No Excel error tokens: metric_recomputation_report.xlsx</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -4744,12 +4744,12 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: model_seed_variance_decomposition.xlsx</t>
+          <t>No Excel error tokens: model_seed_design_audit.xlsx</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
         <is>
-          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E181" s="2" t="inlineStr"/>
@@ -4767,12 +4767,12 @@
       </c>
       <c r="C182" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: remaining_author_actions.xlsx</t>
+          <t>No Excel error tokens: model_seed_results_revised.xlsx</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
-          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E182" s="2" t="inlineStr"/>
@@ -4790,12 +4790,12 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: reviewer_concern_response_revision_location.xlsx</t>
+          <t>No Excel error tokens: model_seed_variance_decomposition.xlsx</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
-          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E183" s="2" t="inlineStr"/>
@@ -4813,12 +4813,12 @@
       </c>
       <c r="C184" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: simulation_negative_result_audit.xlsx</t>
+          <t>No Excel error tokens: remaining_author_actions.xlsx</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
-          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E184" s="2" t="inlineStr"/>
@@ -4836,7 +4836,7 @@
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: submission_remaining_actions.xlsx</t>
+          <t>No Excel error tokens: reviewer_concern_response_revision_location.xlsx</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -4859,12 +4859,12 @@
       </c>
       <c r="C186" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: supplementary_tables_sheet_audit.xlsx</t>
+          <t>No Excel error tokens: simulation_negative_result_audit.xlsx</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
         <is>
-          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=3; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E186" s="2" t="inlineStr"/>
@@ -4882,12 +4882,12 @@
       </c>
       <c r="C187" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: temporal_independence_audit.xlsx</t>
+          <t>No Excel error tokens: submission_remaining_actions.xlsx</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
         <is>
-          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E187" s="2" t="inlineStr"/>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="C188" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: temporal_stress_test_revised.xlsx</t>
+          <t>No Excel error tokens: supplementary_tables_sheet_audit.xlsx</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -4928,12 +4928,12 @@
       </c>
       <c r="C189" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: word_wps_libreoffice_pdf_comparison.xlsx</t>
+          <t>No Excel error tokens: temporal_independence_audit.xlsx</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
         <is>
-          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E189" s="2" t="inlineStr"/>
@@ -4951,12 +4951,12 @@
       </c>
       <c r="C190" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: word_wps_libreoffice_pdf_comparison_strict.xlsx</t>
+          <t>No Excel error tokens: temporal_stress_test_revised.xlsx</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
         <is>
-          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E190" s="2" t="inlineStr"/>
@@ -4974,12 +4974,12 @@
       </c>
       <c r="C191" s="2" t="inlineStr">
         <is>
-          <t>No Excel error tokens: data_dictionary.xlsx</t>
+          <t>No Excel error tokens: word_wps_libreoffice_pdf_comparison.xlsx</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
         <is>
-          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
+          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E191" s="2" t="inlineStr"/>
@@ -4992,17 +4992,17 @@
       </c>
       <c r="B192" s="2" t="inlineStr">
         <is>
-          <t>Reproducibility</t>
+          <t>Spreadsheets</t>
         </is>
       </c>
       <c r="C192" s="2" t="inlineStr">
         <is>
-          <t>Additional file 4 SHA-256 matches</t>
+          <t>No Excel error tokens: word_wps_libreoffice_pdf_comparison_strict.xlsx</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
         <is>
-          <t>actual=10B4385D65337D0919AA5B11344519441CF77DC1C9BB4F56051DADF826501A71; stated=10B4385D65337D0919AA5B11344519441CF77DC1C9BB4F56051DADF826501A71</t>
+          <t>sheets=1; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E192" s="2" t="inlineStr"/>
@@ -5015,17 +5015,17 @@
       </c>
       <c r="B193" s="2" t="inlineStr">
         <is>
-          <t>Reproducibility</t>
+          <t>Spreadsheets</t>
         </is>
       </c>
       <c r="C193" s="2" t="inlineStr">
         <is>
-          <t>Additional file 4 ZIP integrity</t>
+          <t>No Excel error tokens: data_dictionary.xlsx</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
         <is>
-          <t>bad member=None</t>
+          <t>sheets=2; formulas=0; errors=0; cells=[]</t>
         </is>
       </c>
       <c r="E193" s="2" t="inlineStr"/>
@@ -5043,12 +5043,12 @@
       </c>
       <c r="C194" s="2" t="inlineStr">
         <is>
-          <t>Additional file 4 internal SHA-256 manifest</t>
+          <t>Additional file 4 SHA-256 matches</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
         <is>
-          <t>verified=884/884; mismatches=[]</t>
+          <t>actual=10B4385D65337D0919AA5B11344519441CF77DC1C9BB4F56051DADF826501A71; stated=10B4385D65337D0919AA5B11344519441CF77DC1C9BB4F56051DADF826501A71</t>
         </is>
       </c>
       <c r="E194" s="2" t="inlineStr"/>
@@ -5066,12 +5066,12 @@
       </c>
       <c r="C195" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: README.md</t>
+          <t>Additional file 4 ZIP integrity</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=12920</t>
+          <t>bad member=None</t>
         </is>
       </c>
       <c r="E195" s="2" t="inlineStr"/>
@@ -5089,12 +5089,12 @@
       </c>
       <c r="C196" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: VERSION</t>
+          <t>Additional file 4 internal SHA-256 manifest</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=29</t>
+          <t>verified=884/884; mismatches=[]</t>
         </is>
       </c>
       <c r="E196" s="2" t="inlineStr"/>
@@ -5112,12 +5112,12 @@
       </c>
       <c r="C197" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: CITATION.cff</t>
+          <t>Required repository file: README.md</t>
         </is>
       </c>
       <c r="D197" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=318</t>
+          <t>exists=True; bytes=12920</t>
         </is>
       </c>
       <c r="E197" s="2" t="inlineStr"/>
@@ -5135,12 +5135,12 @@
       </c>
       <c r="C198" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: LICENSE</t>
+          <t>Required repository file: VERSION</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=1100</t>
+          <t>exists=True; bytes=29</t>
         </is>
       </c>
       <c r="E198" s="2" t="inlineStr"/>
@@ -5158,12 +5158,12 @@
       </c>
       <c r="C199" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: SHA256SUMS.txt</t>
+          <t>Required repository file: CITATION.cff</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=2176</t>
+          <t>exists=True; bytes=318</t>
         </is>
       </c>
       <c r="E199" s="2" t="inlineStr"/>
@@ -5181,12 +5181,12 @@
       </c>
       <c r="C200" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: environment.yml</t>
+          <t>Required repository file: LICENSE</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=127</t>
+          <t>exists=True; bytes=1100</t>
         </is>
       </c>
       <c r="E200" s="2" t="inlineStr"/>
@@ -5204,12 +5204,12 @@
       </c>
       <c r="C201" s="2" t="inlineStr">
         <is>
-          <t>Required repository file: requirements-lock.txt</t>
+          <t>Required repository file: SHA256SUMS.txt</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
         <is>
-          <t>exists=True; bytes=219</t>
+          <t>exists=True; bytes=2176</t>
         </is>
       </c>
       <c r="E201" s="2" t="inlineStr"/>
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>R12 release/version identified</t>
+          <t>Required repository file: environment.yml</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>R11, R12, paper-release-2026-08-r12</t>
+          <t>exists=True; bytes=127</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr"/>
@@ -5250,12 +5250,12 @@
       </c>
       <c r="C203" s="2" t="inlineStr">
         <is>
-          <t>README has no obsolete Figures 1–7 wording</t>
+          <t>Required repository file: requirements-lock.txt</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
         <is>
-          <t>found=False</t>
+          <t>exists=True; bytes=219</t>
         </is>
       </c>
       <c r="E203" s="2" t="inlineStr"/>
@@ -5273,12 +5273,12 @@
       </c>
       <c r="C204" s="2" t="inlineStr">
         <is>
-          <t>OSI-approved MIT license</t>
+          <t>R12 release/version identified</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>MIT License</t>
+          <t>R11, R12, paper-release-2026-08-r12</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr"/>
@@ -5291,17 +5291,17 @@
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>References</t>
+          <t>Reproducibility</t>
         </is>
       </c>
       <c r="C205" s="2" t="inlineStr">
         <is>
-          <t>Numbered references are sequential</t>
+          <t>README has no obsolete Figures 1–7 wording</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>count=38; first=[1, 2, 3]; last=[36, 37, 38]</t>
+          <t>found=False</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr"/>
@@ -5314,24 +5314,20 @@
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>References</t>
+          <t>Reproducibility</t>
         </is>
       </c>
       <c r="C206" s="2" t="inlineStr">
         <is>
-          <t>DOI presence/structure</t>
+          <t>OSI-approved MIT license</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>DOI-like references=29/38</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>Manual bibliographic verification remains advisable for items without DOI</t>
-        </is>
-      </c>
+          <t>MIT License</t>
+        </is>
+      </c>
+      <c r="E206" s="2" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" s="3" t="inlineStr">
@@ -5346,12 +5342,12 @@
       </c>
       <c r="C207" s="2" t="inlineStr">
         <is>
-          <t>Body URLs limited to ORCID and required software-availability links</t>
+          <t>Numbered references are sequential</t>
         </is>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>permitted=[(8, 'ORCID: Furong Zheng, https://orcid.org/0009-0002-5036-4761'), (146, 'The archived public software release is available at https://github.com/zfr0857/FZYC-Mol/releases/tag/paper-release-2026'), (150, 'Software record. Project name: FZYC-Mol candidate-pool audit. Project homepage: https://github.com/zfr0857/FZYC-Mol. Arc')]; unexpected=[]</t>
+          <t>count=38; first=[1, 2, 3]; last=[36, 37, 38]</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr"/>
@@ -5364,20 +5360,24 @@
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Cross-software</t>
+          <t>References</t>
         </is>
       </c>
       <c r="C208" s="2" t="inlineStr">
         <is>
-          <t>WPS PDF generated</t>
+          <t>DOI presence/structure</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>pages=33; bytes=4585450</t>
-        </is>
-      </c>
-      <c r="E208" s="2" t="inlineStr"/>
+          <t>DOI-like references=29/38</t>
+        </is>
+      </c>
+      <c r="E208" s="2" t="inlineStr">
+        <is>
+          <t>Manual bibliographic verification remains advisable for items without DOI</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="3" t="inlineStr">
@@ -5387,77 +5387,123 @@
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
+          <t>References</t>
+        </is>
+      </c>
+      <c r="C209" s="2" t="inlineStr">
+        <is>
+          <t>Body URLs limited to ORCID and required software-availability links</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>permitted=[(8, 'ORCID: Furong Zheng, https://orcid.org/0009-0002-5036-4761'), (146, 'The archived public software release is available at https://github.com/zfr0857/FZYC-Mol/releases/tag/paper-release-2026'), (150, 'Software record. Project name: FZYC-Mol candidate-pool audit. Project homepage: https://github.com/zfr0857/FZYC-Mol. Arc')]; unexpected=[]</t>
+        </is>
+      </c>
+      <c r="E209" s="2" t="inlineStr"/>
+    </row>
+    <row r="210">
+      <c r="A210" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B210" s="2" t="inlineStr">
+        <is>
           <t>Cross-software</t>
         </is>
       </c>
-      <c r="C209" s="2" t="inlineStr">
+      <c r="C210" s="2" t="inlineStr">
+        <is>
+          <t>WPS PDF generated</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>pages=33; bytes=4585450</t>
+        </is>
+      </c>
+      <c r="E210" s="2" t="inlineStr"/>
+    </row>
+    <row r="211">
+      <c r="A211" s="3" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>Cross-software</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="inlineStr">
         <is>
           <t>LibreOffice PDF generated</t>
         </is>
       </c>
-      <c r="D209" s="2" t="inlineStr">
+      <c r="D211" s="2" t="inlineStr">
         <is>
           <t>pages=34; bytes=2664811</t>
         </is>
       </c>
-      <c r="E209" s="2" t="inlineStr"/>
-    </row>
-    <row r="210">
-      <c r="A210" s="5" t="inlineStr">
+      <c r="E211" s="2" t="inlineStr"/>
+    </row>
+    <row r="212">
+      <c r="A212" s="5" t="inlineStr">
         <is>
           <t>NOT VERIFIED</t>
         </is>
       </c>
-      <c r="B210" s="2" t="inlineStr">
+      <c r="B212" s="2" t="inlineStr">
         <is>
           <t>Cross-software</t>
         </is>
       </c>
-      <c r="C210" s="2" t="inlineStr">
+      <c r="C212" s="2" t="inlineStr">
         <is>
           <t>Microsoft Word PDF</t>
         </is>
       </c>
-      <c r="D210" s="2" t="inlineStr">
+      <c r="D212" s="2" t="inlineStr">
         <is>
           <t>Local Word export has not completed reliably</t>
         </is>
       </c>
-      <c r="E210" s="2" t="inlineStr">
+      <c r="E212" s="2" t="inlineStr">
         <is>
           <t>Open the final DOCX in Word and export PDF before submission</t>
         </is>
       </c>
     </row>
-    <row r="211">
-      <c r="A211" s="5" t="inlineStr">
+    <row r="213">
+      <c r="A213" s="5" t="inlineStr">
         <is>
           <t>NOT VERIFIED</t>
         </is>
       </c>
-      <c r="B211" s="2" t="inlineStr">
+      <c r="B213" s="2" t="inlineStr">
         <is>
           <t>Submission system</t>
         </is>
       </c>
-      <c r="C211" s="2" t="inlineStr">
+      <c r="C213" s="2" t="inlineStr">
         <is>
           <t>Submission preview PDF</t>
         </is>
       </c>
-      <c r="D211" s="2" t="inlineStr">
+      <c r="D213" s="2" t="inlineStr">
         <is>
           <t>Requires author login and upload</t>
         </is>
       </c>
-      <c r="E211" s="2" t="inlineStr">
+      <c r="E213" s="2" t="inlineStr">
         <is>
           <t>Upload all files, inspect the generated preview page by page, and approve only after verification</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E211"/>
+  <autoFilter ref="A1:E213"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5468,7 +5514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:E154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -6414,14 +6460,14 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>6181</v>
+        <v>6184</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>0.006</v>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>4133F3C3D087A95855D6BB9259067BF6CE644C85F1A276224DF1BA5BFD0A0F77</t>
+          <t>49F0288BAF5DBD6F53BE3857A38449122454B0B40721A353AFB2C775E3D9E136</t>
         </is>
       </c>
     </row>
@@ -6743,7 +6789,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>B3035F03CD725DD8C2B4479DC95863E3F612F1086F985B495D14E0E2531C5AB6</t>
+          <t>0C3DCA160BCD2492168EF6B947C9EEE03323BA3A1BE5622F25FB503360C428DB</t>
         </is>
       </c>
     </row>
@@ -6789,37 +6835,37 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>33E17011955A687604FCD3781648CB462643B3FCEC343B9ECD84053C7402CAB5</t>
+          <t>EE986CDB5F57735FA4A8CCD3CCE0BD9D223F1AC6E777B822073FB5595D12CD59</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/full_content_and_format_consistency_audit.xlsx</t>
+          <t>04_Audits_and_source_data/formula_table_and_format_audit_20260815.md</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>7080</v>
+        <v>5455</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.007</v>
+        <v>0.005</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>5C8651F66103BE73731D7314F3C00FBEB2574FD25DA749E7AF9118CB4CBAA0C5</t>
+          <t>E67B94AF46A011EE259CE36D21C8CB7411294A470523BC0EFEC402387B4CA15A</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/journal_format_compliance_audit.xlsx</t>
+          <t>04_Audits_and_source_data/formula_table_and_format_audit_20260815.xlsx</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -6828,44 +6874,44 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>7149</v>
+        <v>8281</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.007</v>
+        <v>0.008</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>9D0B9B6A0966516C76A34746D053C81CF5D642F82F92410FEE7825EED580B2A0</t>
+          <t>88593C6E700E779EBEF57E22EC3AAE8C2FBC29134667B6DA233051FE6DF2D0AE</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_submission_audit_20260810.md</t>
+          <t>04_Audits_and_source_data/full_content_and_format_consistency_audit.xlsx</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C60" s="2" t="n">
-        <v>1338</v>
+        <v>7080</v>
       </c>
       <c r="D60" s="2" t="n">
-        <v>0.001</v>
+        <v>0.007</v>
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>102C77DCA5D15A00F1C49621FC702D7D069ABA8B29D8C9EF6285305C4961946A</t>
+          <t>5C8651F66103BE73731D7314F3C00FBEB2574FD25DA749E7AF9118CB4CBAA0C5</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_submission_audit_20260810.xlsx</t>
+          <t>04_Audits_and_source_data/journal_format_compliance_audit.xlsx</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -6874,136 +6920,136 @@
         </is>
       </c>
       <c r="C61" s="2" t="n">
-        <v>27654</v>
+        <v>7149</v>
       </c>
       <c r="D61" s="2" t="n">
-        <v>0.026</v>
+        <v>0.007</v>
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>9D3A6C7D32B210257121D6F3F7BCB26EBB229C2FD6FE549D85251ABB45A5872D</t>
+          <t>9D0B9B6A0966516C76A34746D053C81CF5D642F82F92410FEE7825EED580B2A0</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_A_source.csv</t>
+          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_audit_20260815.md</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C62" s="2" t="n">
-        <v>2826</v>
+        <v>1111</v>
       </c>
       <c r="D62" s="2" t="n">
-        <v>0.003</v>
+        <v>0.001</v>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>DA901BE96B1FE7EDA5D84A480C11EB9186518934224A407BDA1A86DD0A5B4622</t>
+          <t>D6272F52A050802813D60187F62F6E6ACE3BCEF5FD7144369FC5B16423CB2BD0</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_B_source.csv</t>
+          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_audit_20260815.xlsx</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>1883</v>
+        <v>28198</v>
       </c>
       <c r="D63" s="2" t="n">
-        <v>0.002</v>
+        <v>0.027</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>A9B9A0E488414DA67E8B696035E69FD14E6D4AAEC56EDA7309F7AD6F8D1A9070</t>
+          <t>1A0889D52575F4DED6B6F584EAD3E1831E64A75725F728D928AC9664323AC9B6</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_C_source.csv</t>
+          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_submission_audit_20260810.md</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C64" s="2" t="n">
-        <v>4448</v>
+        <v>1338</v>
       </c>
       <c r="D64" s="2" t="n">
-        <v>0.004</v>
+        <v>0.001</v>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>B32DBB2CFF444D865480D848D2243A6D7F711692F560EA5680BA7C318B8A84B5</t>
+          <t>102C77DCA5D15A00F1C49621FC702D7D069ABA8B29D8C9EF6285305C4961946A</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_D_source.csv</t>
+          <t>04_Audits_and_source_data/Journal_of_Cheminformatics_full_submission_audit_20260810.xlsx</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C65" s="2" t="n">
-        <v>1469</v>
+        <v>27654</v>
       </c>
       <c r="D65" s="2" t="n">
-        <v>0.001</v>
+        <v>0.026</v>
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>0135CFAA1AB66AE6E9540E6F5ADC2B15E3AA0BEEB4F078E0A48313F8BBE33262</t>
+          <t>9D3A6C7D32B210257121D6F3F7BCB26EBB229C2FD6FE549D85251ABB45A5872D</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_source_data.xlsx</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_A_source.csv</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C66" s="2" t="n">
-        <v>13607</v>
+        <v>2826</v>
       </c>
       <c r="D66" s="2" t="n">
-        <v>0.013</v>
+        <v>0.003</v>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>CCFEE7A626AB1A1C993AFF50A7C446867CC03280D4727B20D0298735EC7EDD0D</t>
+          <t>DA901BE96B1FE7EDA5D84A480C11EB9186518934224A407BDA1A86DD0A5B4622</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/audit_gap_decomposition_units.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_B_source.csv</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -7012,21 +7058,21 @@
         </is>
       </c>
       <c r="C67" s="2" t="n">
-        <v>89014</v>
+        <v>1883</v>
       </c>
       <c r="D67" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.002</v>
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>58AA14D12DB69243F8D1BDB5BC0253C8AA956E951B7F98EFE41C5D966F9C4AF5</t>
+          <t>A9B9A0E488414DA67E8B696035E69FD14E6D4AAEC56EDA7309F7AD6F8D1A9070</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/candidate_composition_controls.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_C_source.csv</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -7035,21 +7081,21 @@
         </is>
       </c>
       <c r="C68" s="2" t="n">
-        <v>2597</v>
+        <v>4448</v>
       </c>
       <c r="D68" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>1B17F5137AFA2752B47FC7A31E91C956E5BA7E92EAE75C50465ED7C8AD97F87A</t>
+          <t>B32DBB2CFF444D865480D848D2243A6D7F711692F560EA5680BA7C318B8A84B5</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/classification_metric_selector_comparisons_final.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_Panel_D_source.csv</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -7058,44 +7104,44 @@
         </is>
       </c>
       <c r="C69" s="2" t="n">
-        <v>29163</v>
+        <v>1469</v>
       </c>
       <c r="D69" s="2" t="n">
-        <v>0.028</v>
+        <v>0.001</v>
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>AC77C848D9BA486E8BFCC302E2231EA37235F35ED4D3520C863833F7CB0EBAAF</t>
+          <t>0135CFAA1AB66AE6E9540E6F5ADC2B15E3AA0BEEB4F078E0A48313F8BBE33262</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/cross_fitted_complete_intervals.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/Figure_6_source_data.xlsx</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C70" s="2" t="n">
-        <v>8202</v>
+        <v>13607</v>
       </c>
       <c r="D70" s="2" t="n">
-        <v>0.008</v>
+        <v>0.013</v>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>FDC11FC7206FFF4A68E0E8DBEFCDFAEC89162FADA0C738682660E640B9B66858</t>
+          <t>CCFEE7A626AB1A1C993AFF50A7C446867CC03280D4727B20D0298735EC7EDD0D</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/cross_fitted_fold_effects.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/audit_gap_decomposition_units.csv</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -7104,21 +7150,21 @@
         </is>
       </c>
       <c r="C71" s="2" t="n">
-        <v>10667</v>
+        <v>89014</v>
       </c>
       <c r="D71" s="2" t="n">
-        <v>0.01</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>86C93729849B024402FF896985A84C1E1706B1BB0815D771317567A52F9F49FB</t>
+          <t>58AA14D12DB69243F8D1BDB5BC0253C8AA956E951B7F98EFE41C5D966F9C4AF5</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_bootstrap_5000_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/candidate_composition_controls.csv</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -7127,21 +7173,21 @@
         </is>
       </c>
       <c r="C72" s="2" t="n">
-        <v>211229</v>
+        <v>2597</v>
       </c>
       <c r="D72" s="2" t="n">
-        <v>0.201</v>
+        <v>0.002</v>
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>19F0164A3B12B143B24F511260F49EE7B3D0412FF6DDF4A4DE2BC0898440257E</t>
+          <t>1B17F5137AFA2752B47FC7A31E91C956E5BA7E92EAE75C50465ED7C8AD97F87A</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_leave_one_out.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/classification_metric_selector_comparisons_final.csv</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -7150,21 +7196,21 @@
         </is>
       </c>
       <c r="C73" s="2" t="n">
-        <v>30415</v>
+        <v>29163</v>
       </c>
       <c r="D73" s="2" t="n">
-        <v>0.029</v>
+        <v>0.028</v>
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>A194AB0C2E798F180A9DB35C8DD42A44F9F73E9EEC5821A97576CBB58A45CA03</t>
+          <t>AC77C848D9BA486E8BFCC302E2231EA37235F35ED4D3520C863833F7CB0EBAAF</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_reference_sensitivity.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/cross_fitted_complete_intervals.csv</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
@@ -7173,21 +7219,21 @@
         </is>
       </c>
       <c r="C74" s="2" t="n">
-        <v>46814</v>
+        <v>8202</v>
       </c>
       <c r="D74" s="2" t="n">
-        <v>0.045</v>
+        <v>0.008</v>
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>98872CF4C8047931F9280F8E5B18EB7B40FFB2D07E30F0DC4C7A92A5B2A56078</t>
+          <t>FDC11FC7206FFF4A68E0E8DBEFCDFAEC89162FADA0C738682660E640B9B66858</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_2_seed_level_decomposition_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/cross_fitted_fold_effects.csv</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
@@ -7196,21 +7242,21 @@
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>7519</v>
+        <v>10667</v>
       </c>
       <c r="D75" s="2" t="n">
-        <v>0.007</v>
+        <v>0.01</v>
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>707A1B743C7F876450B938AC451FE672608087B3B6FF78D9FC56E2EE9368F716</t>
+          <t>86C93729849B024402FF896985A84C1E1706B1BB0815D771317567A52F9F49FB</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_5D_integrated_forest_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_bootstrap_5000_summary.csv</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
@@ -7219,21 +7265,21 @@
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>2554</v>
+        <v>211229</v>
       </c>
       <c r="D76" s="2" t="n">
-        <v>0.002</v>
+        <v>0.201</v>
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>A751454FEAED20B9D6FC5C24685060C579A66B301F17C8AB9F005598C7567FBF</t>
+          <t>19F0164A3B12B143B24F511260F49EE7B3D0412FF6DDF4A4DE2BC0898440257E</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8A_double_triangle_matrix_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_leave_one_out.csv</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
@@ -7242,21 +7288,21 @@
         </is>
       </c>
       <c r="C77" s="2" t="n">
-        <v>1020</v>
+        <v>30415</v>
       </c>
       <c r="D77" s="2" t="n">
-        <v>0.001</v>
+        <v>0.029</v>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>C81A877AD91A81A16AA934CB8C1E2F46B35CC8492B1B4DBF026FDE4D91229CD9</t>
+          <t>A194AB0C2E798F180A9DB35C8DD42A44F9F73E9EEC5821A97576CBB58A45CA03</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8A_prediction_diversity_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/effective_rank_reference_sensitivity.csv</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
@@ -7265,21 +7311,21 @@
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>321</v>
+        <v>46814</v>
       </c>
       <c r="D78" s="2" t="n">
-        <v>0</v>
+        <v>0.045</v>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>716256319EC5E74D9690D863F6A47874A39397C9763D6434AF366498CDF7F95C</t>
+          <t>98872CF4C8047931F9280F8E5B18EB7B40FFB2D07E30F0DC4C7A92A5B2A56078</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8B_support_risk_matrix_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_2_seed_level_decomposition_source.csv</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
@@ -7288,21 +7334,21 @@
         </is>
       </c>
       <c r="C79" s="2" t="n">
-        <v>2006</v>
+        <v>7519</v>
       </c>
       <c r="D79" s="2" t="n">
-        <v>0.002</v>
+        <v>0.007</v>
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>67095218C0DD9782BF17A005EE2AFE88C206DC01DD446D00AB3C51DC1B9C7349</t>
+          <t>707A1B743C7F876450B938AC451FE672608087B3B6FF78D9FC56E2EE9368F716</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8C_scaffold_reliability_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_5D_integrated_forest_source.csv</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
@@ -7311,21 +7357,21 @@
         </is>
       </c>
       <c r="C80" s="2" t="n">
-        <v>517</v>
+        <v>2554</v>
       </c>
       <c r="D80" s="2" t="n">
-        <v>0</v>
+        <v>0.002</v>
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>A11AC30CD0FE2775915599179AF2992B988371FCFDBB1C1B579F4D94E82C572A</t>
+          <t>A751454FEAED20B9D6FC5C24685060C579A66B301F17C8AB9F005598C7567FBF</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8D_four_model_clintox_source.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8A_double_triangle_matrix_source.csv</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
@@ -7334,21 +7380,21 @@
         </is>
       </c>
       <c r="C81" s="2" t="n">
-        <v>743</v>
+        <v>1020</v>
       </c>
       <c r="D81" s="2" t="n">
         <v>0.001</v>
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>2A0CC40EF6AC50BF7C37BAEC773CAA70A4FB5D803D7CE33E877A0393A6D3F07C</t>
+          <t>C81A877AD91A81A16AA934CB8C1E2F46B35CC8492B1B4DBF026FDE4D91229CD9</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k3_220_subset_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8A_prediction_diversity_summary.csv</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
@@ -7357,21 +7403,21 @@
         </is>
       </c>
       <c r="C82" s="2" t="n">
-        <v>846607</v>
+        <v>321</v>
       </c>
       <c r="D82" s="2" t="n">
-        <v>0.8070000000000001</v>
+        <v>0</v>
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>976887F7BBC54317660980680B1E01975404FE37283FE3F321682ADDF9BF2148</t>
+          <t>716256319EC5E74D9690D863F6A47874A39397C9763D6434AF366498CDF7F95C</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k3_220_subset_units.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8B_support_risk_matrix_source.csv</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
@@ -7380,21 +7426,21 @@
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>7682775</v>
+        <v>2006</v>
       </c>
       <c r="D83" s="2" t="n">
-        <v>7.327</v>
+        <v>0.002</v>
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>765677E15217853696EAC50F07BB5F4A4A952308B092EA193CF3C0E8BD05773D</t>
+          <t>67095218C0DD9782BF17A005EE2AFE88C206DC01DD446D00AB3C51DC1B9C7349</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k_multiview_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8C_scaffold_reliability_source.csv</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
@@ -7403,21 +7449,21 @@
         </is>
       </c>
       <c r="C84" s="2" t="n">
-        <v>32785</v>
+        <v>517</v>
       </c>
       <c r="D84" s="2" t="n">
-        <v>0.031</v>
+        <v>0</v>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>B23CBE44DFA446F4BDE179547F67E7E50975995309BA9949F6FD129DD99672B4</t>
+          <t>A11AC30CD0FE2775915599179AF2992B988371FCFDBB1C1B579F4D94E82C572A</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/mechanism_permutation_null_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/Figure_8D_four_model_clintox_source.csv</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
@@ -7426,21 +7472,21 @@
         </is>
       </c>
       <c r="C85" s="2" t="n">
-        <v>1160</v>
+        <v>743</v>
       </c>
       <c r="D85" s="2" t="n">
         <v>0.001</v>
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>B9BD13E3716259722BB4D3437E657AD29D2781BEA5674469C750FFB218A5D956</t>
+          <t>2A0CC40EF6AC50BF7C37BAEC773CAA70A4FB5D803D7CE33E877A0393A6D3F07C</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/mechanism_signal_recovery_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k3_220_subset_summary.csv</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
@@ -7449,21 +7495,21 @@
         </is>
       </c>
       <c r="C86" s="2" t="n">
-        <v>4172</v>
+        <v>846607</v>
       </c>
       <c r="D86" s="2" t="n">
-        <v>0.004</v>
+        <v>0.8070000000000001</v>
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>9EF8773B3ACCBB86F9F063C8A7B4471A4CD96C5A6B4EE0D68B56B1FE9DB5EDD2</t>
+          <t>976887F7BBC54317660980680B1E01975404FE37283FE3F321682ADDF9BF2148</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/paper19_oracle_extreme_value_simulation.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k3_220_subset_units.csv</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
@@ -7472,21 +7518,21 @@
         </is>
       </c>
       <c r="C87" s="2" t="n">
-        <v>22022</v>
+        <v>7682775</v>
       </c>
       <c r="D87" s="2" t="n">
-        <v>0.021</v>
+        <v>7.327</v>
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>80A0529B90E4D39AF5E1218E76FA75E80F5C230C86D7615931D2C9875FF8BA00</t>
+          <t>765677E15217853696EAC50F07BB5F4A4A952308B092EA193CF3C0E8BD05773D</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/ranking_metric_main_summary.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/matched_k_multiview_summary.csv</t>
         </is>
       </c>
       <c r="B88" s="2" t="inlineStr">
@@ -7495,67 +7541,67 @@
         </is>
       </c>
       <c r="C88" s="2" t="n">
-        <v>2544</v>
+        <v>32785</v>
       </c>
       <c r="D88" s="2" t="n">
-        <v>0.002</v>
+        <v>0.031</v>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>1E0939602E699CEF988E624ACCEC358D1F24E0ECBA6D5BAEB23A8A50874D48FF</t>
+          <t>B23CBE44DFA446F4BDE179547F67E7E50975995309BA9949F6FD129DD99672B4</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/README.md</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/mechanism_permutation_null_summary.csv</t>
         </is>
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C89" s="2" t="n">
-        <v>1928</v>
+        <v>1160</v>
       </c>
       <c r="D89" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>831195D0E236E3DE8976B4CC8366D60A2839D739209AD2C763A7DF5778DCD662</t>
+          <t>B9BD13E3716259722BB4D3437E657AD29D2781BEA5674469C750FFB218A5D956</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/README.md</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/mechanism_signal_recovery_summary.csv</t>
         </is>
       </c>
       <c r="B90" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C90" s="2" t="n">
-        <v>291</v>
+        <v>4172</v>
       </c>
       <c r="D90" s="2" t="n">
-        <v>0</v>
+        <v>0.004</v>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>C6E8688DA67D012B199BAFB4EDB58564BB9C00A7AE04059719B74B11BF5BD849</t>
+          <t>9EF8773B3ACCBB86F9F063C8A7B4471A4CD96C5A6B4EE0D68B56B1FE9DB5EDD2</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_1.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/paper19_oracle_extreme_value_simulation.csv</t>
         </is>
       </c>
       <c r="B91" s="2" t="inlineStr">
@@ -7564,21 +7610,21 @@
         </is>
       </c>
       <c r="C91" s="2" t="n">
-        <v>423</v>
+        <v>22022</v>
       </c>
       <c r="D91" s="2" t="n">
-        <v>0</v>
+        <v>0.021</v>
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>1323B17ADFD919A113FB2F38972C38787559B6D931CD849A432AE1675CEAF9C8</t>
+          <t>80A0529B90E4D39AF5E1218E76FA75E80F5C230C86D7615931D2C9875FF8BA00</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_2.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/ranking_metric_main_summary.csv</t>
         </is>
       </c>
       <c r="B92" s="2" t="inlineStr">
@@ -7587,67 +7633,67 @@
         </is>
       </c>
       <c r="C92" s="2" t="n">
-        <v>873</v>
+        <v>2544</v>
       </c>
       <c r="D92" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>0F5AD205165E1B4DBCD8D14563AA84386D3729B5C8A6F3EEA5BDDF7C1C773998</t>
+          <t>1E0939602E699CEF988E624ACCEC358D1F24E0ECBA6D5BAEB23A8A50874D48FF</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_3.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_figures/README.md</t>
         </is>
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C93" s="2" t="n">
-        <v>715</v>
+        <v>1928</v>
       </c>
       <c r="D93" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>B81C3FD77677F3B58DB73A1C89E9F8B62CBC53093BE7BE1CB2331B66127267BD</t>
+          <t>831195D0E236E3DE8976B4CC8366D60A2839D739209AD2C763A7DF5778DCD662</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_4.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/README.md</t>
         </is>
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C94" s="2" t="n">
-        <v>1027</v>
+        <v>291</v>
       </c>
       <c r="D94" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>844BA070B0DA2392269A3C57F287233B71F912C58A90E0DA7B82D80A814638B5</t>
+          <t>C6E8688DA67D012B199BAFB4EDB58564BB9C00A7AE04059719B74B11BF5BD849</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/primary_cross_fitted_effects.csv</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_1.csv</t>
         </is>
       </c>
       <c r="B95" s="2" t="inlineStr">
@@ -7656,136 +7702,136 @@
         </is>
       </c>
       <c r="C95" s="2" t="n">
-        <v>1181</v>
+        <v>423</v>
       </c>
       <c r="D95" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>51B77E1C1DBF8B0FA09822C3F67801E545DCA0AB30C89AF39A5B0B4594BA83CD</t>
+          <t>1323B17ADFD919A113FB2F38972C38787559B6D931CD849A432AE1675CEAF9C8</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/machine_readable_source_tables/README.md</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_2.csv</t>
         </is>
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C96" s="2" t="n">
-        <v>299</v>
+        <v>873</v>
       </c>
       <c r="D96" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>9CC981993FC3110C64FA1E6103208BF68FCBEB9A8335E8CE0E33A2DBD5219C51</t>
+          <t>0F5AD205165E1B4DBCD8D14563AA84386D3729B5C8A6F3EEA5BDDF7C1C773998</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/matched_stochastic_registry_results.xlsx</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_3.csv</t>
         </is>
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C97" s="2" t="n">
-        <v>417682</v>
+        <v>715</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>0.398</v>
+        <v>0.001</v>
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>849C998D194172ED1D6EBED9DA326ACE540DCD76883869D36DD2E61D5C662AD5</t>
+          <t>B81C3FD77677F3B58DB73A1C89E9F8B62CBC53093BE7BE1CB2331B66127267BD</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/metric_recomputation_report.xlsx</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/main_tables/Table_4.csv</t>
         </is>
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C98" s="2" t="n">
-        <v>10595</v>
+        <v>1027</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>64D41A540E34B64AEEA748236050B944168D1224D90F6531598B23AC48376FF7</t>
+          <t>844BA070B0DA2392269A3C57F287233B71F912C58A90E0DA7B82D80A814638B5</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/model_seed_design_audit.xlsx</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/primary_cross_fitted_effects.csv</t>
         </is>
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C99" s="2" t="n">
-        <v>68890</v>
+        <v>1181</v>
       </c>
       <c r="D99" s="2" t="n">
-        <v>0.066</v>
+        <v>0.001</v>
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>AFA9AEF94C0FC48A87277C9A15F3DD26A29108636848F3A709ECF99F3CB0AA5C</t>
+          <t>51B77E1C1DBF8B0FA09822C3F67801E545DCA0AB30C89AF39A5B0B4594BA83CD</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/model_seed_results_revised.xlsx</t>
+          <t>04_Audits_and_source_data/machine_readable_source_tables/README.md</t>
         </is>
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C100" s="2" t="n">
-        <v>63596</v>
+        <v>299</v>
       </c>
       <c r="D100" s="2" t="n">
-        <v>0.061</v>
+        <v>0</v>
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>1973D14660802580E5E7C821F529E9B07D311CA121F4D5E33D302555ABB93804</t>
+          <t>9CC981993FC3110C64FA1E6103208BF68FCBEB9A8335E8CE0E33A2DBD5219C51</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/model_seed_variance_decomposition.xlsx</t>
+          <t>04_Audits_and_source_data/matched_stochastic_registry_results.xlsx</t>
         </is>
       </c>
       <c r="B101" s="2" t="inlineStr">
@@ -7794,67 +7840,67 @@
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>82195</v>
+        <v>417682</v>
       </c>
       <c r="D101" s="2" t="n">
-        <v>0.078</v>
+        <v>0.398</v>
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>A0075EE10B232908A21E82511BA4680C896C242E1CCC090597DC8381F322D1F6</t>
+          <t>849C998D194172ED1D6EBED9DA326ACE540DCD76883869D36DD2E61D5C662AD5</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/ooxml_validation_report.txt</t>
+          <t>04_Audits_and_source_data/metric_recomputation_report.xlsx</t>
         </is>
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C102" s="2" t="n">
-        <v>283</v>
+        <v>10595</v>
       </c>
       <c r="D102" s="2" t="n">
-        <v>0</v>
+        <v>0.01</v>
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>9455B6EB1006876A54103EF506CC8536C237D0F0BC2ED33602FB67CD4D21B4B6</t>
+          <t>64D41A540E34B64AEEA748236050B944168D1224D90F6531598B23AC48376FF7</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/pretraining_overlap_limitation.docx</t>
+          <t>04_Audits_and_source_data/model_seed_design_audit.xlsx</t>
         </is>
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>.docx</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C103" s="2" t="n">
-        <v>36948</v>
+        <v>68890</v>
       </c>
       <c r="D103" s="2" t="n">
-        <v>0.035</v>
+        <v>0.066</v>
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>65FE709709834942789EE67DB8B73E6D4D0609E44ED72AC5F7DA4D25843DC292</t>
+          <t>AFA9AEF94C0FC48A87277C9A15F3DD26A29108636848F3A709ECF99F3CB0AA5C</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/remaining_author_actions.xlsx</t>
+          <t>04_Audits_and_source_data/model_seed_results_revised.xlsx</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr">
@@ -7863,21 +7909,21 @@
         </is>
       </c>
       <c r="C104" s="2" t="n">
-        <v>6296</v>
+        <v>63596</v>
       </c>
       <c r="D104" s="2" t="n">
-        <v>0.006</v>
+        <v>0.061</v>
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>E83B5093F8F756641C1B168C5364E53922FF3E3FE4F1A8874AB9A7E3D674E8DD</t>
+          <t>1973D14660802580E5E7C821F529E9B07D311CA121F4D5E33D302555ABB93804</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/reviewer_concern_response_revision_location.xlsx</t>
+          <t>04_Audits_and_source_data/model_seed_variance_decomposition.xlsx</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr">
@@ -7886,90 +7932,90 @@
         </is>
       </c>
       <c r="C105" s="2" t="n">
-        <v>6833</v>
+        <v>82195</v>
       </c>
       <c r="D105" s="2" t="n">
-        <v>0.007</v>
+        <v>0.078</v>
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>076C5F874D97329DCD49EDA555F219908874118630EC4ACB818C44B0E36793AC</t>
+          <t>A0075EE10B232908A21E82511BA4680C896C242E1CCC090597DC8381F322D1F6</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/simulation_interpretation_revised.docx</t>
+          <t>04_Audits_and_source_data/ooxml_validation_report.txt</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>.docx</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="C106" s="2" t="n">
-        <v>36987</v>
+        <v>283</v>
       </c>
       <c r="D106" s="2" t="n">
-        <v>0.035</v>
+        <v>0</v>
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>0857D6CB39578DD8F0DC761E25E901BBF4D1A9FFFF40DBDAA3043A5121B6C317</t>
+          <t>9455B6EB1006876A54103EF506CC8536C237D0F0BC2ED33602FB67CD4D21B4B6</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/simulation_negative_result_audit.xlsx</t>
+          <t>04_Audits_and_source_data/pretraining_overlap_limitation.docx</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.docx</t>
         </is>
       </c>
       <c r="C107" s="2" t="n">
-        <v>27959</v>
+        <v>36948</v>
       </c>
       <c r="D107" s="2" t="n">
-        <v>0.027</v>
+        <v>0.035</v>
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>32733D2417EC55EE19376722B256A537DA8A303E759BBD49422045DAB2488349</t>
+          <t>65FE709709834942789EE67DB8B73E6D4D0609E44ED72AC5F7DA4D25843DC292</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/submission_readiness_report.docx</t>
+          <t>04_Audits_and_source_data/remaining_author_actions.xlsx</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr">
         <is>
-          <t>.docx</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C108" s="2" t="n">
-        <v>39130</v>
+        <v>6296</v>
       </c>
       <c r="D108" s="2" t="n">
-        <v>0.037</v>
+        <v>0.006</v>
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>E4BD782B9FE0FD6A27BB325AE1A6ABEEF1585F9C849CFB8AA7C6B3AA0DEFF601</t>
+          <t>E83B5093F8F756641C1B168C5364E53922FF3E3FE4F1A8874AB9A7E3D674E8DD</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/submission_remaining_actions.xlsx</t>
+          <t>04_Audits_and_source_data/reviewer_concern_response_revision_location.xlsx</t>
         </is>
       </c>
       <c r="B109" s="2" t="inlineStr">
@@ -7978,21 +8024,21 @@
         </is>
       </c>
       <c r="C109" s="2" t="n">
-        <v>5647</v>
+        <v>6833</v>
       </c>
       <c r="D109" s="2" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>86833ECA32904E068E42B60B4FF1AFC9AAF4E7BE83C33FFA1357191BDDCE96C1</t>
+          <t>076C5F874D97329DCD49EDA555F219908874118630EC4ACB818C44B0E36793AC</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/supplementary_material_completeness_report.docx</t>
+          <t>04_Audits_and_source_data/simulation_interpretation_revised.docx</t>
         </is>
       </c>
       <c r="B110" s="2" t="inlineStr">
@@ -8001,21 +8047,21 @@
         </is>
       </c>
       <c r="C110" s="2" t="n">
-        <v>37355</v>
+        <v>36987</v>
       </c>
       <c r="D110" s="2" t="n">
-        <v>0.036</v>
+        <v>0.035</v>
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>4F181EDDF5C9C7A4CF4C8C723411643C5AFE02AAFAC8776DC7635EFE7AD42FF3</t>
+          <t>0857D6CB39578DD8F0DC761E25E901BBF4D1A9FFFF40DBDAA3043A5121B6C317</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/supplementary_tables_sheet_audit.xlsx</t>
+          <t>04_Audits_and_source_data/simulation_negative_result_audit.xlsx</t>
         </is>
       </c>
       <c r="B111" s="2" t="inlineStr">
@@ -8024,90 +8070,90 @@
         </is>
       </c>
       <c r="C111" s="2" t="n">
-        <v>10651</v>
+        <v>27959</v>
       </c>
       <c r="D111" s="2" t="n">
-        <v>0.01</v>
+        <v>0.027</v>
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>613431626D197C631F1707287813A48FDAFCCD068EF2B3E4E3A003263A761A8D</t>
+          <t>32733D2417EC55EE19376722B256A537DA8A303E759BBD49422045DAB2488349</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/temporal_independence_audit.xlsx</t>
+          <t>04_Audits_and_source_data/submission_readiness_report.docx</t>
         </is>
       </c>
       <c r="B112" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.docx</t>
         </is>
       </c>
       <c r="C112" s="2" t="n">
-        <v>7452</v>
+        <v>39130</v>
       </c>
       <c r="D112" s="2" t="n">
-        <v>0.007</v>
+        <v>0.037</v>
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>CB2E29212B6EE7398A52BDC0B07DF2D1FB9C43993321F1AF3FC2CB476D22D1FD</t>
+          <t>E4BD782B9FE0FD6A27BB325AE1A6ABEEF1585F9C849CFB8AA7C6B3AA0DEFF601</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/temporal_overlap_analysis.py</t>
+          <t>04_Audits_and_source_data/submission_remaining_actions.xlsx</t>
         </is>
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C113" s="2" t="n">
-        <v>27301</v>
+        <v>5647</v>
       </c>
       <c r="D113" s="2" t="n">
-        <v>0.026</v>
+        <v>0.005</v>
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>D8208EC35D53CCAD4EE3FFD7129A11CEF680F1C370D7FEFEF08A91F80FE4194A</t>
+          <t>86833ECA32904E068E42B60B4FF1AFC9AAF4E7BE83C33FFA1357191BDDCE96C1</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/temporal_stress_test_revised.xlsx</t>
+          <t>04_Audits_and_source_data/supplementary_material_completeness_report.docx</t>
         </is>
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.docx</t>
         </is>
       </c>
       <c r="C114" s="2" t="n">
-        <v>11217</v>
+        <v>37355</v>
       </c>
       <c r="D114" s="2" t="n">
-        <v>0.011</v>
+        <v>0.036</v>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>AFD18F002710D17B1838786FBAA24ED832389118C32A080A02F061E048CCA4C6</t>
+          <t>4F181EDDF5C9C7A4CF4C8C723411643C5AFE02AAFAC8776DC7635EFE7AD42FF3</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/word_wps_libreoffice_pdf_comparison.xlsx</t>
+          <t>04_Audits_and_source_data/supplementary_tables_sheet_audit.xlsx</t>
         </is>
       </c>
       <c r="B115" s="2" t="inlineStr">
@@ -8116,21 +8162,21 @@
         </is>
       </c>
       <c r="C115" s="2" t="n">
-        <v>5574</v>
+        <v>10651</v>
       </c>
       <c r="D115" s="2" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>E7B1612C1F568FC33EBB6E86DDDE7537CD0AD141B328FAF7A7A34E4EB9C30641</t>
+          <t>613431626D197C631F1707287813A48FDAFCCD068EF2B3E4E3A003263A761A8D</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
         <is>
-          <t>04_Audits_and_source_data/word_wps_libreoffice_pdf_comparison_strict.xlsx</t>
+          <t>04_Audits_and_source_data/temporal_independence_audit.xlsx</t>
         </is>
       </c>
       <c r="B116" s="2" t="inlineStr">
@@ -8139,113 +8185,113 @@
         </is>
       </c>
       <c r="C116" s="2" t="n">
-        <v>5829</v>
+        <v>7452</v>
       </c>
       <c r="D116" s="2" t="n">
-        <v>0.006</v>
+        <v>0.007</v>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>79DF76A44D9EDA341586DB3958FFFF4A0E39902FF0C5F5955E277858CB4923BF</t>
+          <t>CB2E29212B6EE7398A52BDC0B07DF2D1FB9C43993321F1AF3FC2CB476D22D1FD</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/Additional_file_1_supplementary_methods_LibreOffice.pdf</t>
+          <t>04_Audits_and_source_data/temporal_overlap_analysis.py</t>
         </is>
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>.pdf</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C117" s="2" t="n">
-        <v>458680</v>
+        <v>27301</v>
       </c>
       <c r="D117" s="2" t="n">
-        <v>0.437</v>
+        <v>0.026</v>
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>BFFE6C01E3F110B6C77F81FA5E6AC69F682FEC3BBA4B1C363E9F64D0F2B8D578</t>
+          <t>D8208EC35D53CCAD4EE3FFD7129A11CEF680F1C370D7FEFEF08A91F80FE4194A</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
+          <t>04_Audits_and_source_data/temporal_stress_test_revised.xlsx</t>
         </is>
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>.pdf</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C118" s="2" t="n">
-        <v>2664850</v>
+        <v>11217</v>
       </c>
       <c r="D118" s="2" t="n">
-        <v>2.541</v>
+        <v>0.011</v>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>3DCA9BA79030774255BB31A7AAE291A5318E331D527017A306A7BC0FFFDAEE2A</t>
+          <t>AFD18F002710D17B1838786FBAA24ED832389118C32A080A02F061E048CCA4C6</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/WPS/Additional_file_1_supplementary_methods_WPS.pdf</t>
+          <t>04_Audits_and_source_data/word_wps_libreoffice_pdf_comparison.xlsx</t>
         </is>
       </c>
       <c r="B119" s="2" t="inlineStr">
         <is>
-          <t>.pdf</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C119" s="2" t="n">
-        <v>1211228</v>
+        <v>5574</v>
       </c>
       <c r="D119" s="2" t="n">
-        <v>1.155</v>
+        <v>0.005</v>
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>0849E16BC1D6F99662FEDD4FEC8450AF89FBBEE5046616D0F42DCF499ABBD916</t>
+          <t>E7B1612C1F568FC33EBB6E86DDDE7537CD0AD141B328FAF7A7A34E4EB9C30641</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
+          <t>04_Audits_and_source_data/word_wps_libreoffice_pdf_comparison_strict.xlsx</t>
         </is>
       </c>
       <c r="B120" s="2" t="inlineStr">
         <is>
-          <t>.pdf</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C120" s="2" t="n">
-        <v>4585493</v>
+        <v>5826</v>
       </c>
       <c r="D120" s="2" t="n">
-        <v>4.373</v>
+        <v>0.006</v>
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>F5136E01A63F72A38FE9519245A9190443EFF4C3E73A8BDA26C845FE352FE845</t>
+          <t>34D094FE29E03977E6299B4B44FE70B4E4EE6246458DDC29BA501505AD84A74E</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/Additional_file_1_supplementary_methods_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B121" s="2" t="inlineStr">
@@ -8254,21 +8300,21 @@
         </is>
       </c>
       <c r="C121" s="2" t="n">
-        <v>2664811</v>
+        <v>458680</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>2.541</v>
+        <v>0.437</v>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>E3D18D902ABFA43280AF4AEC02A3D7F8BA37E722BC0C0F0F554BF4DDD7AC3954</t>
+          <t>BFFE6C01E3F110B6C77F81FA5E6AC69F682FEC3BBA4B1C363E9F64D0F2B8D578</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -8277,113 +8323,113 @@
         </is>
       </c>
       <c r="C122" s="2" t="n">
-        <v>4585450</v>
+        <v>2664850</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>4.373</v>
+        <v>2.541</v>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>66F734300D72C85DC7006C58F3ED07D3596EFD7D7E837AD5097F13D3624A5787</t>
+          <t>3DCA9BA79030774255BB31A7AAE291A5318E331D527017A306A7BC0FFFDAEE2A</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/01_S24_generation.py</t>
+          <t>05_Compatibility/Formula_Audit_20260815/WPS/Additional_file_1_supplementary_methods_WPS.pdf</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C123" s="2" t="n">
-        <v>3438</v>
+        <v>1211228</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>0.003</v>
+        <v>1.155</v>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>7ACFE842E202415CDD830C6184190CE34AB0D2AB0FF95CC7BEA30B8D98EBFF3B</t>
+          <t>0849E16BC1D6F99662FEDD4FEC8450AF89FBBEE5046616D0F42DCF499ABBD916</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/04_data_cleaning_audit.py</t>
+          <t>05_Compatibility/Formula_Audit_20260815/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>3576</v>
+        <v>4585493</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>0.003</v>
+        <v>4.373</v>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>A3C63EDF4CE813A3F8D2F0DD8C005A376FBBBA3579CE48A53E3922A50D695B75</t>
+          <t>F5136E01A63F72A38FE9519245A9190443EFF4C3E73A8BDA26C845FE352FE845</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/05_scaffold_split_algorithm.py</t>
+          <t>05_Compatibility/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>2626</v>
+        <v>2664811</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>0.003</v>
+        <v>2.541</v>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>4D09FC1477367EC21BFC748E7FAF96AD02411D84E3970F9BF894AEC5718B030F</t>
+          <t>E3D18D902ABFA43280AF4AEC02A3D7F8BA37E722BC0C0F0F554BF4DDD7AC3954</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/08_data_leakage_tests.py</t>
+          <t>05_Compatibility/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>930</v>
+        <v>4585450</v>
       </c>
       <c r="D126" s="2" t="n">
-        <v>0.001</v>
+        <v>4.373</v>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>08E0F2F888C4507045C56FBB46BBE90396196333CE79D95132A81201853CD29D</t>
+          <t>66F734300D72C85DC7006C58F3ED07D3596EFD7D7E837AD5097F13D3624A5787</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_p0p1_figures_20260808.py</t>
+          <t>06_Reproducibility/01_S24_generation.py</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
@@ -8392,21 +8438,21 @@
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>8747</v>
+        <v>3438</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>0A1C3D764AB795CA881499C8BAE476D75C7A3554DA7CC2010B5505C370373A5D</t>
+          <t>7ACFE842E202415CDD830C6184190CE34AB0D2AB0FF95CC7BEA30B8D98EBFF3B</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_paper21_final_figures.py</t>
+          <t>06_Reproducibility/04_data_cleaning_audit.py</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
@@ -8415,21 +8461,21 @@
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>106220</v>
+        <v>3576</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>0.101</v>
+        <v>0.003</v>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>BDBF7B9936C6DDD81E9C28D4A211375712F449DD7056401C892605941E4B83A4</t>
+          <t>A3C63EDF4CE813A3F8D2F0DD8C005A376FBBBA3579CE48A53E3922A50D695B75</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_round2_figures6_8_20260809.py</t>
+          <t>06_Reproducibility/05_scaffold_split_algorithm.py</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -8438,159 +8484,159 @@
         </is>
       </c>
       <c r="C129" s="2" t="n">
-        <v>8747</v>
+        <v>2626</v>
       </c>
       <c r="D129" s="2" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>8D3999B334554A079CE4D5DB522F1E17CB71A0F4F0227125E02DC30C68DBDA9A</t>
+          <t>4D09FC1477367EC21BFC748E7FAF96AD02411D84E3970F9BF894AEC5718B030F</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/candidate_registry.yaml</t>
+          <t>06_Reproducibility/08_data_leakage_tests.py</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
         <is>
-          <t>.yaml</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>736</v>
+        <v>930</v>
       </c>
       <c r="D130" s="2" t="n">
         <v>0.001</v>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>24A984126556E933298A99A110BBFA3F81181B3C5714F6EA02B66790F9169C4B</t>
+          <t>08E0F2F888C4507045C56FBB46BBE90396196333CE79D95132A81201853CD29D</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/CITATION.cff</t>
+          <t>06_Reproducibility/build_p0p1_figures_20260808.py</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
         <is>
-          <t>.cff</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>318</v>
+        <v>8747</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>B167E1F753F5129484BB64A4185E64BB33580FBF1295786FA5210FFC3F9A6B56</t>
+          <t>0A1C3D764AB795CA881499C8BAE476D75C7A3554DA7CC2010B5505C370373A5D</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/CODE_AND_DATA_CONTENTS.csv</t>
+          <t>06_Reproducibility/build_paper21_final_figures.py</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C132" s="2" t="n">
-        <v>2079</v>
+        <v>106220</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>0.002</v>
+        <v>0.101</v>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>83B47F604B6138814924E276F2C31A39272296BFD6567151983BFCEF10DB492F</t>
+          <t>BDBF7B9936C6DDD81E9C28D4A211375712F449DD7056401C892605941E4B83A4</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/data_cleaning.yaml</t>
+          <t>06_Reproducibility/build_round2_figures6_8_20260809.py</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
         <is>
-          <t>.yaml</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C133" s="2" t="n">
-        <v>639</v>
+        <v>8747</v>
       </c>
       <c r="D133" s="2" t="n">
-        <v>0.001</v>
+        <v>0.008</v>
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>5175A6DF16AF9FE05554C719F56E667E6F8F41DAECC9033168940A2092B39C5B</t>
+          <t>8D3999B334554A079CE4D5DB522F1E17CB71A0F4F0227125E02DC30C68DBDA9A</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/data_dictionary.xlsx</t>
+          <t>06_Reproducibility/candidate_registry.yaml</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.yaml</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>10554</v>
+        <v>736</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>0.01</v>
+        <v>0.001</v>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>0BE4FCC1B707053BB3BC483B4A6FF1062296A3B48113D85A09CBC818032D343B</t>
+          <t>24A984126556E933298A99A110BBFA3F81181B3C5714F6EA02B66790F9169C4B</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/environment.yml</t>
+          <t>06_Reproducibility/CITATION.cff</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>.yml</t>
+          <t>.cff</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
-        <v>127</v>
+        <v>318</v>
       </c>
       <c r="D135" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>D559FBA9E6483242DAFBEC32D44DB89A6F497BEF789C0CBB95D2BFB3D0A7BF70</t>
+          <t>B167E1F753F5129484BB64A4185E64BB33580FBF1295786FA5210FFC3F9A6B56</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/Equation_to_code_mapping.csv</t>
+          <t>06_Reproducibility/CODE_AND_DATA_CONTENTS.csv</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
@@ -8599,333 +8645,425 @@
         </is>
       </c>
       <c r="C136" s="2" t="n">
-        <v>2470</v>
+        <v>2079</v>
       </c>
       <c r="D136" s="2" t="n">
         <v>0.002</v>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>C009641B7C9DB492A61E25E25F4AE04F2E52C92A8094ED8A08779348C4E668C3</t>
+          <t>83B47F604B6138814924E276F2C31A39272296BFD6567151983BFCEF10DB492F</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/file_hash_manifest.csv</t>
+          <t>06_Reproducibility/data_cleaning.yaml</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.yaml</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
-        <v>2083</v>
+        <v>639</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>45F111529A5F4B2E5F219248F6604AEC4632AF4AD391188D3C3AD35CC46B193E</t>
+          <t>5175A6DF16AF9FE05554C719F56E667E6F8F41DAECC9033168940A2092B39C5B</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/FORMULA_SPECIFICATION.md</t>
+          <t>06_Reproducibility/data_dictionary.xlsx</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
-        <v>2204</v>
+        <v>10554</v>
       </c>
       <c r="D138" s="2" t="n">
-        <v>0.002</v>
+        <v>0.01</v>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>27A335B5AE75B5820758C24667C53A90227EE933CD03A8D4A845440E9A164A53</t>
+          <t>0BE4FCC1B707053BB3BC483B4A6FF1062296A3B48113D85A09CBC818032D343B</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/LICENSE</t>
-        </is>
-      </c>
-      <c r="B139" s="2" t="inlineStr"/>
+          <t>06_Reproducibility/environment.yml</t>
+        </is>
+      </c>
+      <c r="B139" s="2" t="inlineStr">
+        <is>
+          <t>.yml</t>
+        </is>
+      </c>
       <c r="C139" s="2" t="n">
-        <v>1100</v>
+        <v>127</v>
       </c>
       <c r="D139" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>28219DC877B61F27CCBDA12120CF898A0CB9B51DFE320E13F47F95D1E083F4AA</t>
+          <t>D559FBA9E6483242DAFBEC32D44DB89A6F497BEF789C0CBB95D2BFB3D0A7BF70</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/README.md</t>
+          <t>06_Reproducibility/Equation_to_code_mapping.csv</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
-        <v>12920</v>
+        <v>2470</v>
       </c>
       <c r="D140" s="2" t="n">
-        <v>0.012</v>
+        <v>0.002</v>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>0FA50D6BFCA5EDA70A01726FF00A397016CA95B24D7F0B3ED9078FFAACBFB609</t>
+          <t>C009641B7C9DB492A61E25E25F4AE04F2E52C92A8094ED8A08779348C4E668C3</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/rebuild_final_figures_6_8_20260809.py</t>
+          <t>06_Reproducibility/file_hash_manifest.csv</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
-        <v>11642</v>
+        <v>2083</v>
       </c>
       <c r="D141" s="2" t="n">
-        <v>0.011</v>
+        <v>0.002</v>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>784149D1B34EA20CA1401775B5A0EFD683DCEB07DB624E8E2A91490F3B536251</t>
+          <t>45F111529A5F4B2E5F219248F6604AEC4632AF4AD391188D3C3AD35CC46B193E</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/redraw_figure1_core_detailed_20260803.py</t>
+          <t>06_Reproducibility/FORMULA_SPECIFICATION.md</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
-        <v>13507</v>
+        <v>2204</v>
       </c>
       <c r="D142" s="2" t="n">
-        <v>0.013</v>
+        <v>0.002</v>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>B84A85E90425E7B9957EDACAC645402A0D44107C2DDA3EDC469E55A8481BE5E4</t>
+          <t>27A335B5AE75B5820758C24667C53A90227EE933CD03A8D4A845440E9A164A53</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/reproducibility_readme.md</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
-        <is>
-          <t>.md</t>
-        </is>
-      </c>
+          <t>06_Reproducibility/LICENSE</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr"/>
       <c r="C143" s="2" t="n">
-        <v>12439</v>
+        <v>1100</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>0.012</v>
+        <v>0.001</v>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>594EB43F12A5B5242859B3D95E3A22E7835FFB41565EACB147715D444243245A</t>
+          <t>28219DC877B61F27CCBDA12120CF898A0CB9B51DFE320E13F47F95D1E083F4AA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/requirements-lock.txt</t>
+          <t>06_Reproducibility/README.md</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C144" s="2" t="n">
-        <v>219</v>
+        <v>12920</v>
       </c>
       <c r="D144" s="2" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
+          <t>0FA50D6BFCA5EDA70A01726FF00A397016CA95B24D7F0B3ED9078FFAACBFB609</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/requirements.txt</t>
+          <t>06_Reproducibility/rebuild_final_figures_6_8_20260809.py</t>
         </is>
       </c>
       <c r="B145" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C145" s="2" t="n">
-        <v>219</v>
+        <v>11642</v>
       </c>
       <c r="D145" s="2" t="n">
-        <v>0</v>
+        <v>0.011</v>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
+          <t>784149D1B34EA20CA1401775B5A0EFD683DCEB07DB624E8E2A91490F3B536251</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/SHA256SUMS.txt</t>
+          <t>06_Reproducibility/redraw_figure1_core_detailed_20260803.py</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
-        <v>2176</v>
+        <v>13507</v>
       </c>
       <c r="D146" s="2" t="n">
-        <v>0.002</v>
+        <v>0.013</v>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>92EE41F691CFD346421233F9DB62977A2EF61E79ED8462D351E8F67FCDC98EAD</t>
+          <t>B84A85E90425E7B9957EDACAC645402A0D44107C2DDA3EDC469E55A8481BE5E4</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/VERSION</t>
-        </is>
-      </c>
-      <c r="B147" s="2" t="inlineStr"/>
+          <t>06_Reproducibility/reproducibility_readme.md</t>
+        </is>
+      </c>
+      <c r="B147" s="2" t="inlineStr">
+        <is>
+          <t>.md</t>
+        </is>
+      </c>
       <c r="C147" s="2" t="n">
-        <v>29</v>
+        <v>12439</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>552CD3B80513860523F64DA50D7EE38D79605BF661502C81EFBC21057AF07CC1</t>
+          <t>594EB43F12A5B5242859B3D95E3A22E7835FFB41565EACB147715D444243245A</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>07_Author_reference_only/Chinese_author_reference_topic_synchronized_R12.9.docx</t>
+          <t>06_Reproducibility/requirements-lock.txt</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>.docx</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
-        <v>5903197</v>
+        <v>219</v>
       </c>
       <c r="D148" s="2" t="n">
-        <v>5.63</v>
+        <v>0</v>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>8B83F2F2760C1E7D6595C7921D8DE0121F041C30C02CAD07371E68C07C3DDC19</t>
+          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>07_Author_reference_only/README_NOT_FOR_SUBMISSION.md</t>
+          <t>06_Reproducibility/requirements.txt</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
-        <v>767</v>
+        <v>219</v>
       </c>
       <c r="D149" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>238B2594ACF1E4912F264D528A737CEA9D95B259D5ADAB21423EDCCCB69F3DFB</t>
+          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
+          <t>06_Reproducibility/SHA256SUMS.txt</t>
+        </is>
+      </c>
+      <c r="B150" s="2" t="inlineStr">
+        <is>
+          <t>.txt</t>
+        </is>
+      </c>
+      <c r="C150" s="2" t="n">
+        <v>2176</v>
+      </c>
+      <c r="D150" s="2" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>92EE41F691CFD346421233F9DB62977A2EF61E79ED8462D351E8F67FCDC98EAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>06_Reproducibility/VERSION</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr"/>
+      <c r="C151" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="D151" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E151" s="2" t="inlineStr">
+        <is>
+          <t>552CD3B80513860523F64DA50D7EE38D79605BF661502C81EFBC21057AF07CC1</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>07_Author_reference_only/Chinese_author_reference_topic_synchronized_R12.9.docx</t>
+        </is>
+      </c>
+      <c r="B152" s="2" t="inlineStr">
+        <is>
+          <t>.docx</t>
+        </is>
+      </c>
+      <c r="C152" s="2" t="n">
+        <v>5903197</v>
+      </c>
+      <c r="D152" s="2" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="E152" s="2" t="inlineStr">
+        <is>
+          <t>8B83F2F2760C1E7D6595C7921D8DE0121F041C30C02CAD07371E68C07C3DDC19</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>07_Author_reference_only/README_NOT_FOR_SUBMISSION.md</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr">
+        <is>
+          <t>.md</t>
+        </is>
+      </c>
+      <c r="C153" s="2" t="n">
+        <v>767</v>
+      </c>
+      <c r="D153" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E153" s="2" t="inlineStr">
+        <is>
+          <t>238B2594ACF1E4912F264D528A737CEA9D95B259D5ADAB21423EDCCCB69F3DFB</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
           <t>DELIVERY_README.md</t>
         </is>
       </c>
-      <c r="B150" s="2" t="inlineStr">
+      <c r="B154" s="2" t="inlineStr">
         <is>
           <t>.md</t>
         </is>
       </c>
-      <c r="C150" s="2" t="n">
+      <c r="C154" s="2" t="n">
         <v>4663</v>
       </c>
-      <c r="D150" s="2" t="n">
+      <c r="D154" s="2" t="n">
         <v>0.004</v>
       </c>
-      <c r="E150" s="2" t="inlineStr">
+      <c r="E154" s="2" t="inlineStr">
         <is>
           <t>ED7FAED56E51848D4F0FC5C449E98A7F90CEDAC9D1F88A479A2F80AB965437D6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E150"/>
+  <autoFilter ref="A1:E154"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Standardize manuscript formula notation and rendering
</commit_message>
<xml_diff>
--- a/submission_documents/audits/Journal_of_Cheminformatics_full_audit_20260815.xlsx
+++ b/submission_documents/audits/Journal_of_Cheminformatics_full_audit_20260815.xlsx
@@ -13,7 +13,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$E$213</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'File inventory'!$A$1:$E$154</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'File inventory'!$A$1:$E$156</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="4">
@@ -5514,7 +5514,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E154"/>
+  <dimension ref="A1:E156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -5609,14 +5609,14 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>5897995</v>
+        <v>5898068</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>5.625</v>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>C29B9CB4FFB95FDC84C51958D285F0474A5478BA77554152E445F68038ACCB89</t>
+          <t>CA5ACE72B1231B0C0BC54DB68AB44AFAA65437F37E21832BD9B47AC92315F2DE</t>
         </is>
       </c>
     </row>
@@ -5678,14 +5678,14 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>44883</v>
+        <v>45096</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>0.043</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>2AFDFD48ABC1ABA827B6AB2FAA1C7DC6CDFEABAC1C7EF47C2DDE2A8DC21C3AA0</t>
+          <t>643A74CD2EA0B8D53C86E038CE1E49382C89010BF2ABC9819E90B100C973ED09</t>
         </is>
       </c>
     </row>
@@ -6851,14 +6851,14 @@
         </is>
       </c>
       <c r="C58" s="2" t="n">
-        <v>5455</v>
+        <v>7117</v>
       </c>
       <c r="D58" s="2" t="n">
-        <v>0.005</v>
+        <v>0.007</v>
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>E67B94AF46A011EE259CE36D21C8CB7411294A470523BC0EFEC402387B4CA15A</t>
+          <t>E1D4340A532DB705FA81BB3DEAC3C40A55CFD67B1F800FD47D4CE46033C13E13</t>
         </is>
       </c>
     </row>
@@ -6874,14 +6874,14 @@
         </is>
       </c>
       <c r="C59" s="2" t="n">
-        <v>8281</v>
+        <v>9121</v>
       </c>
       <c r="D59" s="2" t="n">
-        <v>0.008</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>88593C6E700E779EBEF57E22EC3AAE8C2FBC29134667B6DA233051FE6DF2D0AE</t>
+          <t>71F14008D721C7E18568115DD59321FB1688887802F5E8DD790A64A2ECCFBDDB</t>
         </is>
       </c>
     </row>
@@ -6950,7 +6950,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>D6272F52A050802813D60187F62F6E6ACE3BCEF5FD7144369FC5B16423CB2BD0</t>
+          <t>FA738167F840DF9FEFAC89935406831A1CB16162749763E082CA51C31D67B952</t>
         </is>
       </c>
     </row>
@@ -6966,14 +6966,14 @@
         </is>
       </c>
       <c r="C63" s="2" t="n">
-        <v>28198</v>
+        <v>28567</v>
       </c>
       <c r="D63" s="2" t="n">
         <v>0.027</v>
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>1A0889D52575F4DED6B6F584EAD3E1831E64A75725F728D928AC9664323AC9B6</t>
+          <t>478A91E10EDB9C71803C98F8A2CA4A88DF1037B1B94574E29D35FF26DFBC65A5</t>
         </is>
       </c>
     </row>
@@ -8300,21 +8300,21 @@
         </is>
       </c>
       <c r="C121" s="2" t="n">
-        <v>458680</v>
+        <v>458853</v>
       </c>
       <c r="D121" s="2" t="n">
-        <v>0.437</v>
+        <v>0.438</v>
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>BFFE6C01E3F110B6C77F81FA5E6AC69F682FEC3BBA4B1C363E9F64D0F2B8D578</t>
+          <t>F451D203B02BEBC251021E5030BE5F13D314A848E19D6FD74762833870815F57</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/Chinese_author_reference_topic_synchronized_R12.9_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B122" s="2" t="inlineStr">
@@ -8323,21 +8323,21 @@
         </is>
       </c>
       <c r="C122" s="2" t="n">
-        <v>2664850</v>
+        <v>2984732</v>
       </c>
       <c r="D122" s="2" t="n">
-        <v>2.541</v>
+        <v>2.846</v>
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>3DCA9BA79030774255BB31A7AAE291A5318E331D527017A306A7BC0FFFDAEE2A</t>
+          <t>0417BD0FA5896A1CBAD39421EF292D30EFC3F70106580A2999BC3BB6AB6652A6</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/WPS/Additional_file_1_supplementary_methods_WPS.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B123" s="2" t="inlineStr">
@@ -8346,21 +8346,21 @@
         </is>
       </c>
       <c r="C123" s="2" t="n">
-        <v>1211228</v>
+        <v>2664716</v>
       </c>
       <c r="D123" s="2" t="n">
-        <v>1.155</v>
+        <v>2.541</v>
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>0849E16BC1D6F99662FEDD4FEC8450AF89FBBEE5046616D0F42DCF499ABBD916</t>
+          <t>F795AFDB74BA12F406B6404520D54AA53D329FC3CD3665BA4483CD040DA35A36</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/Formula_Audit_20260815/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/WPS/Additional_file_1_supplementary_methods_WPS.pdf</t>
         </is>
       </c>
       <c r="B124" s="2" t="inlineStr">
@@ -8369,21 +8369,21 @@
         </is>
       </c>
       <c r="C124" s="2" t="n">
-        <v>4585493</v>
+        <v>1211560</v>
       </c>
       <c r="D124" s="2" t="n">
-        <v>4.373</v>
+        <v>1.155</v>
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>F5136E01A63F72A38FE9519245A9190443EFF4C3E73A8BDA26C845FE352FE845</t>
+          <t>A8DCF1F770F23E5E8060DE5F176CF8DC69124ABCE590CFEDAF95A294F07173B8</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/WPS/Chinese_author_reference_topic_synchronized_R12.9_WPS.pdf</t>
         </is>
       </c>
       <c r="B125" s="2" t="inlineStr">
@@ -8392,21 +8392,21 @@
         </is>
       </c>
       <c r="C125" s="2" t="n">
-        <v>2664811</v>
+        <v>4687029</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>2.541</v>
+        <v>4.47</v>
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>E3D18D902ABFA43280AF4AEC02A3D7F8BA37E722BC0C0F0F554BF4DDD7AC3954</t>
+          <t>B1DFAE9C76F22F8E809317DA4F685AB741CDC6881C96738D0D38F1F143875DB5</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
         <is>
-          <t>05_Compatibility/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
+          <t>05_Compatibility/Formula_Audit_20260815/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
         </is>
       </c>
       <c r="B126" s="2" t="inlineStr">
@@ -8415,67 +8415,67 @@
         </is>
       </c>
       <c r="C126" s="2" t="n">
-        <v>4585450</v>
+        <v>4585349</v>
       </c>
       <c r="D126" s="2" t="n">
         <v>4.373</v>
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>66F734300D72C85DC7006C58F3ED07D3596EFD7D7E837AD5097F13D3624A5787</t>
+          <t>5CE7BA3996D983E4A554072A1CCC26CAAA3257A139629ECE1B87F767A34EB6F3</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/01_S24_generation.py</t>
+          <t>05_Compatibility/LibreOffice/manuscript_revised_submission_ready_LibreOffice.pdf</t>
         </is>
       </c>
       <c r="B127" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C127" s="2" t="n">
-        <v>3438</v>
+        <v>2664811</v>
       </c>
       <c r="D127" s="2" t="n">
-        <v>0.003</v>
+        <v>2.541</v>
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>7ACFE842E202415CDD830C6184190CE34AB0D2AB0FF95CC7BEA30B8D98EBFF3B</t>
+          <t>E3D18D902ABFA43280AF4AEC02A3D7F8BA37E722BC0C0F0F554BF4DDD7AC3954</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/04_data_cleaning_audit.py</t>
+          <t>05_Compatibility/WPS/manuscript_revised_submission_ready_WPS.pdf</t>
         </is>
       </c>
       <c r="B128" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.pdf</t>
         </is>
       </c>
       <c r="C128" s="2" t="n">
-        <v>3576</v>
+        <v>4585450</v>
       </c>
       <c r="D128" s="2" t="n">
-        <v>0.003</v>
+        <v>4.373</v>
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>A3C63EDF4CE813A3F8D2F0DD8C005A376FBBBA3579CE48A53E3922A50D695B75</t>
+          <t>66F734300D72C85DC7006C58F3ED07D3596EFD7D7E837AD5097F13D3624A5787</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/05_scaffold_split_algorithm.py</t>
+          <t>06_Reproducibility/01_S24_generation.py</t>
         </is>
       </c>
       <c r="B129" s="2" t="inlineStr">
@@ -8484,21 +8484,21 @@
         </is>
       </c>
       <c r="C129" s="2" t="n">
-        <v>2626</v>
+        <v>3438</v>
       </c>
       <c r="D129" s="2" t="n">
         <v>0.003</v>
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>4D09FC1477367EC21BFC748E7FAF96AD02411D84E3970F9BF894AEC5718B030F</t>
+          <t>7ACFE842E202415CDD830C6184190CE34AB0D2AB0FF95CC7BEA30B8D98EBFF3B</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/08_data_leakage_tests.py</t>
+          <t>06_Reproducibility/04_data_cleaning_audit.py</t>
         </is>
       </c>
       <c r="B130" s="2" t="inlineStr">
@@ -8507,21 +8507,21 @@
         </is>
       </c>
       <c r="C130" s="2" t="n">
-        <v>930</v>
+        <v>3576</v>
       </c>
       <c r="D130" s="2" t="n">
-        <v>0.001</v>
+        <v>0.003</v>
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>08E0F2F888C4507045C56FBB46BBE90396196333CE79D95132A81201853CD29D</t>
+          <t>A3C63EDF4CE813A3F8D2F0DD8C005A376FBBBA3579CE48A53E3922A50D695B75</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_p0p1_figures_20260808.py</t>
+          <t>06_Reproducibility/05_scaffold_split_algorithm.py</t>
         </is>
       </c>
       <c r="B131" s="2" t="inlineStr">
@@ -8530,21 +8530,21 @@
         </is>
       </c>
       <c r="C131" s="2" t="n">
-        <v>8747</v>
+        <v>2626</v>
       </c>
       <c r="D131" s="2" t="n">
-        <v>0.008</v>
+        <v>0.003</v>
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>0A1C3D764AB795CA881499C8BAE476D75C7A3554DA7CC2010B5505C370373A5D</t>
+          <t>4D09FC1477367EC21BFC748E7FAF96AD02411D84E3970F9BF894AEC5718B030F</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_paper21_final_figures.py</t>
+          <t>06_Reproducibility/08_data_leakage_tests.py</t>
         </is>
       </c>
       <c r="B132" s="2" t="inlineStr">
@@ -8553,21 +8553,21 @@
         </is>
       </c>
       <c r="C132" s="2" t="n">
-        <v>106220</v>
+        <v>930</v>
       </c>
       <c r="D132" s="2" t="n">
-        <v>0.101</v>
+        <v>0.001</v>
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>BDBF7B9936C6DDD81E9C28D4A211375712F449DD7056401C892605941E4B83A4</t>
+          <t>08E0F2F888C4507045C56FBB46BBE90396196333CE79D95132A81201853CD29D</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/build_round2_figures6_8_20260809.py</t>
+          <t>06_Reproducibility/build_p0p1_figures_20260808.py</t>
         </is>
       </c>
       <c r="B133" s="2" t="inlineStr">
@@ -8583,240 +8583,244 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>8D3999B334554A079CE4D5DB522F1E17CB71A0F4F0227125E02DC30C68DBDA9A</t>
+          <t>0A1C3D764AB795CA881499C8BAE476D75C7A3554DA7CC2010B5505C370373A5D</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/candidate_registry.yaml</t>
+          <t>06_Reproducibility/build_paper21_final_figures.py</t>
         </is>
       </c>
       <c r="B134" s="2" t="inlineStr">
         <is>
-          <t>.yaml</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C134" s="2" t="n">
-        <v>736</v>
+        <v>106220</v>
       </c>
       <c r="D134" s="2" t="n">
-        <v>0.001</v>
+        <v>0.101</v>
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>24A984126556E933298A99A110BBFA3F81181B3C5714F6EA02B66790F9169C4B</t>
+          <t>BDBF7B9936C6DDD81E9C28D4A211375712F449DD7056401C892605941E4B83A4</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/CITATION.cff</t>
+          <t>06_Reproducibility/build_round2_figures6_8_20260809.py</t>
         </is>
       </c>
       <c r="B135" s="2" t="inlineStr">
         <is>
-          <t>.cff</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C135" s="2" t="n">
-        <v>318</v>
+        <v>8747</v>
       </c>
       <c r="D135" s="2" t="n">
-        <v>0</v>
+        <v>0.008</v>
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>B167E1F753F5129484BB64A4185E64BB33580FBF1295786FA5210FFC3F9A6B56</t>
+          <t>8D3999B334554A079CE4D5DB522F1E17CB71A0F4F0227125E02DC30C68DBDA9A</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/CODE_AND_DATA_CONTENTS.csv</t>
+          <t>06_Reproducibility/candidate_registry.yaml</t>
         </is>
       </c>
       <c r="B136" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.yaml</t>
         </is>
       </c>
       <c r="C136" s="2" t="n">
-        <v>2079</v>
+        <v>736</v>
       </c>
       <c r="D136" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>83B47F604B6138814924E276F2C31A39272296BFD6567151983BFCEF10DB492F</t>
+          <t>24A984126556E933298A99A110BBFA3F81181B3C5714F6EA02B66790F9169C4B</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/data_cleaning.yaml</t>
+          <t>06_Reproducibility/CITATION.cff</t>
         </is>
       </c>
       <c r="B137" s="2" t="inlineStr">
         <is>
-          <t>.yaml</t>
+          <t>.cff</t>
         </is>
       </c>
       <c r="C137" s="2" t="n">
-        <v>639</v>
+        <v>318</v>
       </c>
       <c r="D137" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>5175A6DF16AF9FE05554C719F56E667E6F8F41DAECC9033168940A2092B39C5B</t>
+          <t>B167E1F753F5129484BB64A4185E64BB33580FBF1295786FA5210FFC3F9A6B56</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/data_dictionary.xlsx</t>
+          <t>06_Reproducibility/CODE_AND_DATA_CONTENTS.csv</t>
         </is>
       </c>
       <c r="B138" s="2" t="inlineStr">
         <is>
-          <t>.xlsx</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C138" s="2" t="n">
-        <v>10554</v>
+        <v>2079</v>
       </c>
       <c r="D138" s="2" t="n">
-        <v>0.01</v>
+        <v>0.002</v>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>0BE4FCC1B707053BB3BC483B4A6FF1062296A3B48113D85A09CBC818032D343B</t>
+          <t>83B47F604B6138814924E276F2C31A39272296BFD6567151983BFCEF10DB492F</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/environment.yml</t>
+          <t>06_Reproducibility/data_cleaning.yaml</t>
         </is>
       </c>
       <c r="B139" s="2" t="inlineStr">
         <is>
-          <t>.yml</t>
+          <t>.yaml</t>
         </is>
       </c>
       <c r="C139" s="2" t="n">
-        <v>127</v>
+        <v>639</v>
       </c>
       <c r="D139" s="2" t="n">
-        <v>0</v>
+        <v>0.001</v>
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>D559FBA9E6483242DAFBEC32D44DB89A6F497BEF789C0CBB95D2BFB3D0A7BF70</t>
+          <t>5175A6DF16AF9FE05554C719F56E667E6F8F41DAECC9033168940A2092B39C5B</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/Equation_to_code_mapping.csv</t>
+          <t>06_Reproducibility/data_dictionary.xlsx</t>
         </is>
       </c>
       <c r="B140" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.xlsx</t>
         </is>
       </c>
       <c r="C140" s="2" t="n">
-        <v>2470</v>
+        <v>10554</v>
       </c>
       <c r="D140" s="2" t="n">
-        <v>0.002</v>
+        <v>0.01</v>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>C009641B7C9DB492A61E25E25F4AE04F2E52C92A8094ED8A08779348C4E668C3</t>
+          <t>0BE4FCC1B707053BB3BC483B4A6FF1062296A3B48113D85A09CBC818032D343B</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/file_hash_manifest.csv</t>
+          <t>06_Reproducibility/environment.yml</t>
         </is>
       </c>
       <c r="B141" s="2" t="inlineStr">
         <is>
-          <t>.csv</t>
+          <t>.yml</t>
         </is>
       </c>
       <c r="C141" s="2" t="n">
-        <v>2083</v>
+        <v>127</v>
       </c>
       <c r="D141" s="2" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>45F111529A5F4B2E5F219248F6604AEC4632AF4AD391188D3C3AD35CC46B193E</t>
+          <t>D559FBA9E6483242DAFBEC32D44DB89A6F497BEF789C0CBB95D2BFB3D0A7BF70</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/FORMULA_SPECIFICATION.md</t>
+          <t>06_Reproducibility/Equation_to_code_mapping.csv</t>
         </is>
       </c>
       <c r="B142" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.csv</t>
         </is>
       </c>
       <c r="C142" s="2" t="n">
-        <v>2204</v>
+        <v>2470</v>
       </c>
       <c r="D142" s="2" t="n">
         <v>0.002</v>
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>27A335B5AE75B5820758C24667C53A90227EE933CD03A8D4A845440E9A164A53</t>
+          <t>C009641B7C9DB492A61E25E25F4AE04F2E52C92A8094ED8A08779348C4E668C3</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/LICENSE</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr"/>
+          <t>06_Reproducibility/file_hash_manifest.csv</t>
+        </is>
+      </c>
+      <c r="B143" s="2" t="inlineStr">
+        <is>
+          <t>.csv</t>
+        </is>
+      </c>
       <c r="C143" s="2" t="n">
-        <v>1100</v>
+        <v>2083</v>
       </c>
       <c r="D143" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>28219DC877B61F27CCBDA12120CF898A0CB9B51DFE320E13F47F95D1E083F4AA</t>
+          <t>45F111529A5F4B2E5F219248F6604AEC4632AF4AD391188D3C3AD35CC46B193E</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/README.md</t>
+          <t>06_Reproducibility/FORMULA_SPECIFICATION.md</t>
         </is>
       </c>
       <c r="B144" s="2" t="inlineStr">
@@ -8825,136 +8829,132 @@
         </is>
       </c>
       <c r="C144" s="2" t="n">
-        <v>12920</v>
+        <v>2366</v>
       </c>
       <c r="D144" s="2" t="n">
-        <v>0.012</v>
+        <v>0.002</v>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>0FA50D6BFCA5EDA70A01726FF00A397016CA95B24D7F0B3ED9078FFAACBFB609</t>
+          <t>2C6E5535EF52D45FE535ADEC0689FC45C9347E8CB9B4D289EBCAF54421AFDDD1</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/rebuild_final_figures_6_8_20260809.py</t>
-        </is>
-      </c>
-      <c r="B145" s="2" t="inlineStr">
-        <is>
-          <t>.py</t>
-        </is>
-      </c>
+          <t>06_Reproducibility/LICENSE</t>
+        </is>
+      </c>
+      <c r="B145" s="2" t="inlineStr"/>
       <c r="C145" s="2" t="n">
-        <v>11642</v>
+        <v>1100</v>
       </c>
       <c r="D145" s="2" t="n">
-        <v>0.011</v>
+        <v>0.001</v>
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>784149D1B34EA20CA1401775B5A0EFD683DCEB07DB624E8E2A91490F3B536251</t>
+          <t>28219DC877B61F27CCBDA12120CF898A0CB9B51DFE320E13F47F95D1E083F4AA</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/redraw_figure1_core_detailed_20260803.py</t>
+          <t>06_Reproducibility/README.md</t>
         </is>
       </c>
       <c r="B146" s="2" t="inlineStr">
         <is>
-          <t>.py</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C146" s="2" t="n">
-        <v>13507</v>
+        <v>12920</v>
       </c>
       <c r="D146" s="2" t="n">
-        <v>0.013</v>
+        <v>0.012</v>
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>B84A85E90425E7B9957EDACAC645402A0D44107C2DDA3EDC469E55A8481BE5E4</t>
+          <t>0FA50D6BFCA5EDA70A01726FF00A397016CA95B24D7F0B3ED9078FFAACBFB609</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/reproducibility_readme.md</t>
+          <t>06_Reproducibility/rebuild_final_figures_6_8_20260809.py</t>
         </is>
       </c>
       <c r="B147" s="2" t="inlineStr">
         <is>
-          <t>.md</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C147" s="2" t="n">
-        <v>12439</v>
+        <v>11642</v>
       </c>
       <c r="D147" s="2" t="n">
-        <v>0.012</v>
+        <v>0.011</v>
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>594EB43F12A5B5242859B3D95E3A22E7835FFB41565EACB147715D444243245A</t>
+          <t>784149D1B34EA20CA1401775B5A0EFD683DCEB07DB624E8E2A91490F3B536251</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/requirements-lock.txt</t>
+          <t>06_Reproducibility/redraw_figure1_core_detailed_20260803.py</t>
         </is>
       </c>
       <c r="B148" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.py</t>
         </is>
       </c>
       <c r="C148" s="2" t="n">
-        <v>219</v>
+        <v>13507</v>
       </c>
       <c r="D148" s="2" t="n">
-        <v>0</v>
+        <v>0.013</v>
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
+          <t>B84A85E90425E7B9957EDACAC645402A0D44107C2DDA3EDC469E55A8481BE5E4</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/requirements.txt</t>
+          <t>06_Reproducibility/reproducibility_readme.md</t>
         </is>
       </c>
       <c r="B149" s="2" t="inlineStr">
         <is>
-          <t>.txt</t>
+          <t>.md</t>
         </is>
       </c>
       <c r="C149" s="2" t="n">
-        <v>219</v>
+        <v>12439</v>
       </c>
       <c r="D149" s="2" t="n">
-        <v>0</v>
+        <v>0.012</v>
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
+          <t>594EB43F12A5B5242859B3D95E3A22E7835FFB41565EACB147715D444243245A</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/SHA256SUMS.txt</t>
+          <t>06_Reproducibility/requirements-lock.txt</t>
         </is>
       </c>
       <c r="B150" s="2" t="inlineStr">
@@ -8963,107 +8963,153 @@
         </is>
       </c>
       <c r="C150" s="2" t="n">
-        <v>2176</v>
+        <v>219</v>
       </c>
       <c r="D150" s="2" t="n">
-        <v>0.002</v>
+        <v>0</v>
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>92EE41F691CFD346421233F9DB62977A2EF61E79ED8462D351E8F67FCDC98EAD</t>
+          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
         <is>
-          <t>06_Reproducibility/VERSION</t>
-        </is>
-      </c>
-      <c r="B151" s="2" t="inlineStr"/>
+          <t>06_Reproducibility/requirements.txt</t>
+        </is>
+      </c>
+      <c r="B151" s="2" t="inlineStr">
+        <is>
+          <t>.txt</t>
+        </is>
+      </c>
       <c r="C151" s="2" t="n">
-        <v>29</v>
+        <v>219</v>
       </c>
       <c r="D151" s="2" t="n">
         <v>0</v>
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>552CD3B80513860523F64DA50D7EE38D79605BF661502C81EFBC21057AF07CC1</t>
+          <t>FC76CEAEB5526DE5A55DE6CBC9D3196757B9A6C19BFFF4659E07C6CCEA678C40</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
         <is>
-          <t>07_Author_reference_only/Chinese_author_reference_topic_synchronized_R12.9.docx</t>
+          <t>06_Reproducibility/SHA256SUMS.txt</t>
         </is>
       </c>
       <c r="B152" s="2" t="inlineStr">
         <is>
-          <t>.docx</t>
+          <t>.txt</t>
         </is>
       </c>
       <c r="C152" s="2" t="n">
-        <v>5903197</v>
+        <v>2176</v>
       </c>
       <c r="D152" s="2" t="n">
-        <v>5.63</v>
+        <v>0.002</v>
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>8B83F2F2760C1E7D6595C7921D8DE0121F041C30C02CAD07371E68C07C3DDC19</t>
+          <t>92EE41F691CFD346421233F9DB62977A2EF61E79ED8462D351E8F67FCDC98EAD</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
         <is>
-          <t>07_Author_reference_only/README_NOT_FOR_SUBMISSION.md</t>
-        </is>
-      </c>
-      <c r="B153" s="2" t="inlineStr">
-        <is>
-          <t>.md</t>
-        </is>
-      </c>
+          <t>06_Reproducibility/VERSION</t>
+        </is>
+      </c>
+      <c r="B153" s="2" t="inlineStr"/>
       <c r="C153" s="2" t="n">
-        <v>767</v>
+        <v>29</v>
       </c>
       <c r="D153" s="2" t="n">
-        <v>0.001</v>
+        <v>0</v>
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>238B2594ACF1E4912F264D528A737CEA9D95B259D5ADAB21423EDCCCB69F3DFB</t>
+          <t>552CD3B80513860523F64DA50D7EE38D79605BF661502C81EFBC21057AF07CC1</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
         <is>
+          <t>07_Author_reference_only/Chinese_author_reference_topic_synchronized_R12.9.docx</t>
+        </is>
+      </c>
+      <c r="B154" s="2" t="inlineStr">
+        <is>
+          <t>.docx</t>
+        </is>
+      </c>
+      <c r="C154" s="2" t="n">
+        <v>5903242</v>
+      </c>
+      <c r="D154" s="2" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="E154" s="2" t="inlineStr">
+        <is>
+          <t>605D04EE929332FE56810024490FF274A158CF0BEE9B747F3A9E8FAF31932823</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>07_Author_reference_only/README_NOT_FOR_SUBMISSION.md</t>
+        </is>
+      </c>
+      <c r="B155" s="2" t="inlineStr">
+        <is>
+          <t>.md</t>
+        </is>
+      </c>
+      <c r="C155" s="2" t="n">
+        <v>767</v>
+      </c>
+      <c r="D155" s="2" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>238B2594ACF1E4912F264D528A737CEA9D95B259D5ADAB21423EDCCCB69F3DFB</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
           <t>DELIVERY_README.md</t>
         </is>
       </c>
-      <c r="B154" s="2" t="inlineStr">
+      <c r="B156" s="2" t="inlineStr">
         <is>
           <t>.md</t>
         </is>
       </c>
-      <c r="C154" s="2" t="n">
+      <c r="C156" s="2" t="n">
         <v>4663</v>
       </c>
-      <c r="D154" s="2" t="n">
+      <c r="D156" s="2" t="n">
         <v>0.004</v>
       </c>
-      <c r="E154" s="2" t="inlineStr">
+      <c r="E156" s="2" t="inlineStr">
         <is>
           <t>ED7FAED56E51848D4F0FC5C449E98A7F90CEDAC9D1F88A479A2F80AB965437D6</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E154"/>
+  <autoFilter ref="A1:E156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>